<commit_message>
weird bug but all works
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t xml:space="preserve">polymer</t>
   </si>
@@ -93,12 +93,6 @@
   </si>
   <si>
     <t xml:space="preserve">Rayon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lyocell</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modal</t>
   </si>
 </sst>
 </file>
@@ -4707,546 +4701,6 @@
         <v>1520.21158912113</v>
       </c>
     </row>
-    <row r="215">
-      <c r="A215" t="s">
-        <v>26</v>
-      </c>
-      <c r="B215" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C215" t="s">
-        <v>7</v>
-      </c>
-      <c r="D215" t="n">
-        <v>0.0833836187095184</v>
-      </c>
-      <c r="E215" t="n">
-        <v>5.65744205749315</v>
-      </c>
-      <c r="F215" t="n">
-        <v>1520.00017701984</v>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="s">
-        <v>26</v>
-      </c>
-      <c r="B216" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C216" t="s">
-        <v>8</v>
-      </c>
-      <c r="D216" t="n">
-        <v>0.0999882782178372</v>
-      </c>
-      <c r="E216" t="n">
-        <v>5.86836376380892</v>
-      </c>
-      <c r="F216" t="n">
-        <v>1520.00017701984</v>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="s">
-        <v>26</v>
-      </c>
-      <c r="B217" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C217" t="s">
-        <v>7</v>
-      </c>
-      <c r="D217" t="n">
-        <v>0.300307606749357</v>
-      </c>
-      <c r="E217" t="n">
-        <v>14.2190355045313</v>
-      </c>
-      <c r="F217" t="n">
-        <v>1519.99997437236</v>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="s">
-        <v>27</v>
-      </c>
-      <c r="B218" t="n">
-        <v>1</v>
-      </c>
-      <c r="C218" t="s">
-        <v>7</v>
-      </c>
-      <c r="D218" t="n">
-        <v>0.000000814243945492164</v>
-      </c>
-      <c r="E218" t="n">
-        <v>0.0000675333540085995</v>
-      </c>
-      <c r="F218" t="n">
-        <v>2495.39160987973</v>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="s">
-        <v>27</v>
-      </c>
-      <c r="B219" t="n">
-        <v>1</v>
-      </c>
-      <c r="C219" t="s">
-        <v>8</v>
-      </c>
-      <c r="D219" t="n">
-        <v>0.00000392409821565979</v>
-      </c>
-      <c r="E219" t="n">
-        <v>0.000325411097308621</v>
-      </c>
-      <c r="F219" t="n">
-        <v>2495.39160987973</v>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="s">
-        <v>27</v>
-      </c>
-      <c r="B220" t="n">
-        <v>1</v>
-      </c>
-      <c r="C220" t="s">
-        <v>9</v>
-      </c>
-      <c r="D220" t="n">
-        <v>0.000115738843203759</v>
-      </c>
-      <c r="E220" t="n">
-        <v>0.00938789759014455</v>
-      </c>
-      <c r="F220" t="n">
-        <v>2495.39160987973</v>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="s">
-        <v>27</v>
-      </c>
-      <c r="B221" t="n">
-        <v>10</v>
-      </c>
-      <c r="C221" t="s">
-        <v>7</v>
-      </c>
-      <c r="D221" t="n">
-        <v>0.0000369297389419497</v>
-      </c>
-      <c r="E221" t="n">
-        <v>0.00464464650697526</v>
-      </c>
-      <c r="F221" t="n">
-        <v>1677.63151784358</v>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="s">
-        <v>27</v>
-      </c>
-      <c r="B222" t="n">
-        <v>10</v>
-      </c>
-      <c r="C222" t="s">
-        <v>8</v>
-      </c>
-      <c r="D222" t="n">
-        <v>0.000110973174010516</v>
-      </c>
-      <c r="E222" t="n">
-        <v>0.0138403679984313</v>
-      </c>
-      <c r="F222" t="n">
-        <v>1677.63151784358</v>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="s">
-        <v>27</v>
-      </c>
-      <c r="B223" t="n">
-        <v>10</v>
-      </c>
-      <c r="C223" t="s">
-        <v>9</v>
-      </c>
-      <c r="D223" t="n">
-        <v>0.0035584983102518</v>
-      </c>
-      <c r="E223" t="n">
-        <v>0.270351129154867</v>
-      </c>
-      <c r="F223" t="n">
-        <v>1677.63151784358</v>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="s">
-        <v>27</v>
-      </c>
-      <c r="B224" t="n">
-        <v>100</v>
-      </c>
-      <c r="C224" t="s">
-        <v>7</v>
-      </c>
-      <c r="D224" t="n">
-        <v>0.00259874561631262</v>
-      </c>
-      <c r="E224" t="n">
-        <v>0.367976804774418</v>
-      </c>
-      <c r="F224" t="n">
-        <v>1500.21590878229</v>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="s">
-        <v>27</v>
-      </c>
-      <c r="B225" t="n">
-        <v>100</v>
-      </c>
-      <c r="C225" t="s">
-        <v>8</v>
-      </c>
-      <c r="D225" t="n">
-        <v>0.00665108847531712</v>
-      </c>
-      <c r="E225" t="n">
-        <v>0.718785598237358</v>
-      </c>
-      <c r="F225" t="n">
-        <v>1500.21590878229</v>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="s">
-        <v>27</v>
-      </c>
-      <c r="B226" t="n">
-        <v>100</v>
-      </c>
-      <c r="C226" t="s">
-        <v>9</v>
-      </c>
-      <c r="D226" t="n">
-        <v>0.0316442191859101</v>
-      </c>
-      <c r="E226" t="n">
-        <v>1.78556984839564</v>
-      </c>
-      <c r="F226" t="n">
-        <v>1500.21590878229</v>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="s">
-        <v>27</v>
-      </c>
-      <c r="B227" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C227" t="s">
-        <v>7</v>
-      </c>
-      <c r="D227" t="n">
-        <v>0.0812096588938284</v>
-      </c>
-      <c r="E227" t="n">
-        <v>5.61246192144937</v>
-      </c>
-      <c r="F227" t="n">
-        <v>1500.00018179589</v>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="s">
-        <v>27</v>
-      </c>
-      <c r="B228" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C228" t="s">
-        <v>8</v>
-      </c>
-      <c r="D228" t="n">
-        <v>0.0976007054511689</v>
-      </c>
-      <c r="E228" t="n">
-        <v>5.82682840147347</v>
-      </c>
-      <c r="F228" t="n">
-        <v>1500.00018179589</v>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" t="s">
-        <v>27</v>
-      </c>
-      <c r="B229" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C229" t="s">
-        <v>7</v>
-      </c>
-      <c r="D229" t="n">
-        <v>0.294296882202111</v>
-      </c>
-      <c r="E229" t="n">
-        <v>14.1306412246364</v>
-      </c>
-      <c r="F229" t="n">
-        <v>1499.99997476641</v>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" t="s">
-        <v>28</v>
-      </c>
-      <c r="B230" t="n">
-        <v>1</v>
-      </c>
-      <c r="C230" t="s">
-        <v>7</v>
-      </c>
-      <c r="D230" t="n">
-        <v>0.000000814294058988281</v>
-      </c>
-      <c r="E230" t="n">
-        <v>0.0000676360198760847</v>
-      </c>
-      <c r="F230" t="n">
-        <v>2495.48377577483</v>
-      </c>
-    </row>
-    <row r="231">
-      <c r="A231" t="s">
-        <v>28</v>
-      </c>
-      <c r="B231" t="n">
-        <v>1</v>
-      </c>
-      <c r="C231" t="s">
-        <v>8</v>
-      </c>
-      <c r="D231" t="n">
-        <v>0.00000392433972210361</v>
-      </c>
-      <c r="E231" t="n">
-        <v>0.000325905681476606</v>
-      </c>
-      <c r="F231" t="n">
-        <v>2495.48377577483</v>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" t="s">
-        <v>28</v>
-      </c>
-      <c r="B232" t="n">
-        <v>1</v>
-      </c>
-      <c r="C232" t="s">
-        <v>9</v>
-      </c>
-      <c r="D232" t="n">
-        <v>0.000115745916655048</v>
-      </c>
-      <c r="E232" t="n">
-        <v>0.00940186572120423</v>
-      </c>
-      <c r="F232" t="n">
-        <v>2495.48377577483</v>
-      </c>
-    </row>
-    <row r="233">
-      <c r="A233" t="s">
-        <v>28</v>
-      </c>
-      <c r="B233" t="n">
-        <v>10</v>
-      </c>
-      <c r="C233" t="s">
-        <v>7</v>
-      </c>
-      <c r="D233" t="n">
-        <v>0.0000378230618969218</v>
-      </c>
-      <c r="E233" t="n">
-        <v>0.00470603672293593</v>
-      </c>
-      <c r="F233" t="n">
-        <v>1694.07888566558</v>
-      </c>
-    </row>
-    <row r="234">
-      <c r="A234" t="s">
-        <v>28</v>
-      </c>
-      <c r="B234" t="n">
-        <v>10</v>
-      </c>
-      <c r="C234" t="s">
-        <v>8</v>
-      </c>
-      <c r="D234" t="n">
-        <v>0.000113652714049356</v>
-      </c>
-      <c r="E234" t="n">
-        <v>0.0140219586818437</v>
-      </c>
-      <c r="F234" t="n">
-        <v>1694.07888566558</v>
-      </c>
-    </row>
-    <row r="235">
-      <c r="A235" t="s">
-        <v>28</v>
-      </c>
-      <c r="B235" t="n">
-        <v>10</v>
-      </c>
-      <c r="C235" t="s">
-        <v>9</v>
-      </c>
-      <c r="D235" t="n">
-        <v>0.00362887240316199</v>
-      </c>
-      <c r="E235" t="n">
-        <v>0.272901540334341</v>
-      </c>
-      <c r="F235" t="n">
-        <v>1694.07888566558</v>
-      </c>
-    </row>
-    <row r="236">
-      <c r="A236" t="s">
-        <v>28</v>
-      </c>
-      <c r="B236" t="n">
-        <v>100</v>
-      </c>
-      <c r="C236" t="s">
-        <v>7</v>
-      </c>
-      <c r="D236" t="n">
-        <v>0.00269888569222591</v>
-      </c>
-      <c r="E236" t="n">
-        <v>0.372338530680835</v>
-      </c>
-      <c r="F236" t="n">
-        <v>1520.21158912113</v>
-      </c>
-    </row>
-    <row r="237">
-      <c r="A237" t="s">
-        <v>28</v>
-      </c>
-      <c r="B237" t="n">
-        <v>100</v>
-      </c>
-      <c r="C237" t="s">
-        <v>8</v>
-      </c>
-      <c r="D237" t="n">
-        <v>0.00688512295406375</v>
-      </c>
-      <c r="E237" t="n">
-        <v>0.726058568902636</v>
-      </c>
-      <c r="F237" t="n">
-        <v>1520.21158912113</v>
-      </c>
-    </row>
-    <row r="238">
-      <c r="A238" t="s">
-        <v>28</v>
-      </c>
-      <c r="B238" t="n">
-        <v>100</v>
-      </c>
-      <c r="C238" t="s">
-        <v>9</v>
-      </c>
-      <c r="D238" t="n">
-        <v>0.0323903661003693</v>
-      </c>
-      <c r="E238" t="n">
-        <v>1.79775130323394</v>
-      </c>
-      <c r="F238" t="n">
-        <v>1520.21158912113</v>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" t="s">
-        <v>28</v>
-      </c>
-      <c r="B239" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C239" t="s">
-        <v>7</v>
-      </c>
-      <c r="D239" t="n">
-        <v>0.0833836187095184</v>
-      </c>
-      <c r="E239" t="n">
-        <v>5.65744205749315</v>
-      </c>
-      <c r="F239" t="n">
-        <v>1520.00017701984</v>
-      </c>
-    </row>
-    <row r="240">
-      <c r="A240" t="s">
-        <v>28</v>
-      </c>
-      <c r="B240" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C240" t="s">
-        <v>8</v>
-      </c>
-      <c r="D240" t="n">
-        <v>0.0999882782178372</v>
-      </c>
-      <c r="E240" t="n">
-        <v>5.86836376380892</v>
-      </c>
-      <c r="F240" t="n">
-        <v>1520.00017701984</v>
-      </c>
-    </row>
-    <row r="241">
-      <c r="A241" t="s">
-        <v>28</v>
-      </c>
-      <c r="B241" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C241" t="s">
-        <v>7</v>
-      </c>
-      <c r="D241" t="n">
-        <v>0.300307606749357</v>
-      </c>
-      <c r="E241" t="n">
-        <v>14.2190355045313</v>
-      </c>
-      <c r="F241" t="n">
-        <v>1519.99997437236</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>